<commit_message>
refactor(engine): implementa sniffer dinâmico no parser e blindagem contra KeyError no Streamlit
</commit_message>
<xml_diff>
--- a/data/output/audit_relatorio_bruto.txt.xlsx
+++ b/data/output/audit_relatorio_bruto.txt.xlsx
@@ -554,7 +554,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="51" customWidth="1" min="8" max="8"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -787,11 +787,11 @@
         <v>1</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>ZERO_VALUE_TRANSACTION, FUTURE_DATE_TRANSACTION</t>
+          <t>ZERO_VALUE_TRANSACTION</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">

</xml_diff>